<commit_message>
Sprint 2.2 - Added Department Generator
Sprint 2.2 - Added Department Generator
</commit_message>
<xml_diff>
--- a/Data/Master/Company.xlsx
+++ b/Data/Master/Company.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Company" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,6 +443,276 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NS001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Nova Manufacturing</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Manufacturing</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NS002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Nova Retail</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NS003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Nova Digital</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Digital</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NS004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Nova Services</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NS005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Nova Logistics</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Logistics</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NS006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Nova Healthcare</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NS007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Nova Energy</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>NS008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Nova Foods</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>NS009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Nova Finance</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>NS010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Nova International</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>